<commit_message>
Generated output file from workflow
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -551,12 +551,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>23 days, 20:22:26.808971</t>
+          <t>22 days, 20:19:00.984271</t>
         </is>
       </c>
     </row>
@@ -604,12 +604,12 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>23 days, 3:22:26.808847</t>
+          <t>22 days, 3:19:00.984147</t>
         </is>
       </c>
     </row>
@@ -718,12 +718,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>23 days, 2:22:26.808806</t>
+          <t>22 days, 2:19:00.984101</t>
         </is>
       </c>
     </row>
@@ -775,12 +775,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>23 days, 2:22:26.808772</t>
+          <t>22 days, 2:19:00.984059</t>
         </is>
       </c>
     </row>
@@ -832,12 +832,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>23 days, 2:22:26.808740</t>
+          <t>22 days, 2:19:00.984013</t>
         </is>
       </c>
     </row>
@@ -889,12 +889,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>23 days, 2:22:26.808709</t>
+          <t>22 days, 2:19:00.983973</t>
         </is>
       </c>
     </row>
@@ -946,12 +946,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>23 days, 2:22:26.808676</t>
+          <t>22 days, 2:19:00.983931</t>
         </is>
       </c>
     </row>
@@ -1003,12 +1003,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>23 days, 2:22:26.808608</t>
+          <t>22 days, 2:19:00.983892</t>
         </is>
       </c>
     </row>
@@ -1060,12 +1060,12 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>23 days, 2:22:26.808565</t>
+          <t>22 days, 2:19:00.983823</t>
         </is>
       </c>
     </row>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808533</t>
+          <t>22 days, 2:04:00.983779</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1174,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808501</t>
+          <t>22 days, 2:04:00.983741</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1231,12 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808469</t>
+          <t>22 days, 2:04:00.983703</t>
         </is>
       </c>
     </row>
@@ -1288,12 +1288,12 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808438</t>
+          <t>22 days, 2:04:00.983664</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808409</t>
+          <t>22 days, 2:04:00.983628</t>
         </is>
       </c>
     </row>
@@ -1402,12 +1402,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808378</t>
+          <t>22 days, 2:04:00.983592</t>
         </is>
       </c>
     </row>
@@ -1459,12 +1459,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808347</t>
+          <t>22 days, 2:04:00.983555</t>
         </is>
       </c>
     </row>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808317</t>
+          <t>22 days, 2:04:00.983519</t>
         </is>
       </c>
     </row>
@@ -1573,12 +1573,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808288</t>
+          <t>22 days, 2:04:00.983483</t>
         </is>
       </c>
     </row>
@@ -1630,12 +1630,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808258</t>
+          <t>22 days, 2:04:00.983448</t>
         </is>
       </c>
     </row>
@@ -1687,12 +1687,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>23 days, 2:07:26.808228</t>
+          <t>22 days, 2:04:00.983412</t>
         </is>
       </c>
     </row>
@@ -1749,12 +1749,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>23 days, 1:37:26.808198</t>
+          <t>22 days, 1:34:00.983375</t>
         </is>
       </c>
     </row>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>23 days, 1:37:26.808168</t>
+          <t>22 days, 1:34:00.983339</t>
         </is>
       </c>
     </row>
@@ -1873,12 +1873,12 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>23 days, 1:37:26.808135</t>
+          <t>22 days, 1:34:00.983299</t>
         </is>
       </c>
     </row>
@@ -1935,12 +1935,12 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>23 days, 1:37:26.808101</t>
+          <t>22 days, 1:34:00.983259</t>
         </is>
       </c>
     </row>
@@ -1997,12 +1997,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>23 days, 1:37:26.808069</t>
+          <t>22 days, 1:34:00.983219</t>
         </is>
       </c>
     </row>
@@ -2050,12 +2050,12 @@
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2103,12 +2103,12 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2160,12 +2160,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>19 days, 20:22:26.807968</t>
+          <t>18 days, 20:19:00.983100</t>
         </is>
       </c>
     </row>
@@ -2217,12 +2217,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>19 days, 5:22:26.807938</t>
+          <t>18 days, 5:19:00.983062</t>
         </is>
       </c>
     </row>
@@ -2274,12 +2274,12 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>19 days, 5:22:26.807909</t>
+          <t>18 days, 5:19:00.983027</t>
         </is>
       </c>
     </row>
@@ -2331,12 +2331,12 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>19 days, 5:22:26.807882</t>
+          <t>18 days, 5:19:00.982993</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2437,12 +2437,12 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2494,12 +2494,12 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>19 days, 4:22:26.807793</t>
+          <t>18 days, 4:19:00.982886</t>
         </is>
       </c>
     </row>
@@ -2551,12 +2551,12 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>18 days, 22:22:26.807762</t>
+          <t>17 days, 22:19:00.982824</t>
         </is>
       </c>
     </row>
@@ -2604,12 +2604,12 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2662,12 +2662,12 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2719,12 +2719,12 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>17 days, 23:52:26.807683</t>
+          <t>16 days, 23:49:00.982720</t>
         </is>
       </c>
     </row>
@@ -2772,12 +2772,12 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2825,12 +2825,12 @@
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2878,12 +2878,12 @@
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2931,12 +2931,12 @@
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -2980,12 +2980,12 @@
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3037,12 +3037,12 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>17 days, 22:07:26.807522</t>
+          <t>16 days, 22:04:00.982537</t>
         </is>
       </c>
     </row>
@@ -3090,12 +3090,12 @@
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3143,12 +3143,12 @@
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3200,12 +3200,12 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>17 days, 22:07:26.807442</t>
+          <t>16 days, 22:04:00.982439</t>
         </is>
       </c>
     </row>
@@ -3253,12 +3253,12 @@
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3306,12 +3306,12 @@
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3359,12 +3359,12 @@
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3412,12 +3412,12 @@
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3465,12 +3465,12 @@
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3518,12 +3518,12 @@
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3571,12 +3571,12 @@
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3628,12 +3628,12 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>17 days, 20:22:26.807230</t>
+          <t>16 days, 20:19:00.982190</t>
         </is>
       </c>
     </row>
@@ -3685,12 +3685,12 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>17 days, 20:22:26.807196</t>
+          <t>16 days, 20:19:00.982154</t>
         </is>
       </c>
     </row>
@@ -3742,12 +3742,12 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>17 days, 20:22:26.807161</t>
+          <t>16 days, 20:19:00.982116</t>
         </is>
       </c>
     </row>
@@ -3799,12 +3799,12 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>17 days, 20:22:26.807131</t>
+          <t>16 days, 20:19:00.982080</t>
         </is>
       </c>
     </row>
@@ -3852,12 +3852,12 @@
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3905,12 +3905,12 @@
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -3958,12 +3958,12 @@
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4011,12 +4011,12 @@
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4064,12 +4064,12 @@
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4117,12 +4117,12 @@
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4170,12 +4170,12 @@
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4223,12 +4223,12 @@
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4276,12 +4276,12 @@
       <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4329,12 +4329,12 @@
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4386,12 +4386,12 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>17 days, 20:22:26.806843</t>
+          <t>16 days, 20:19:00.981719</t>
         </is>
       </c>
     </row>
@@ -4443,12 +4443,12 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>17 days, 20:22:26.806811</t>
+          <t>16 days, 20:19:00.981673</t>
         </is>
       </c>
     </row>
@@ -4496,12 +4496,12 @@
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4549,12 +4549,12 @@
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4602,12 +4602,12 @@
       <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4655,12 +4655,12 @@
       <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4708,12 +4708,12 @@
       <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4761,12 +4761,12 @@
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4814,12 +4814,12 @@
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4867,12 +4867,12 @@
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -4924,12 +4924,12 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>17 days, 20:22:26.806555</t>
+          <t>16 days, 20:19:00.981380</t>
         </is>
       </c>
     </row>
@@ -4977,12 +4977,12 @@
       <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5030,12 +5030,12 @@
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5083,12 +5083,12 @@
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5136,12 +5136,12 @@
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5189,12 +5189,12 @@
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5242,12 +5242,12 @@
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5295,12 +5295,12 @@
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5348,12 +5348,12 @@
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5410,12 +5410,12 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>17 days, 5:52:26.806317</t>
+          <t>16 days, 5:49:00.981092</t>
         </is>
       </c>
     </row>
@@ -5472,12 +5472,12 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>17 days, 5:52:26.806291</t>
+          <t>16 days, 5:49:00.981058</t>
         </is>
       </c>
     </row>
@@ -5525,12 +5525,12 @@
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5578,12 +5578,12 @@
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5631,12 +5631,12 @@
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5684,12 +5684,12 @@
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5737,12 +5737,12 @@
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5790,12 +5790,12 @@
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5843,12 +5843,12 @@
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5901,12 +5901,12 @@
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -5959,12 +5959,12 @@
       <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6012,12 +6012,12 @@
       <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6065,12 +6065,12 @@
       <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6118,12 +6118,12 @@
       <c r="J103" t="inlineStr"/>
       <c r="K103" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6171,12 +6171,12 @@
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6224,12 +6224,12 @@
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6277,12 +6277,12 @@
       <c r="J106" t="inlineStr"/>
       <c r="K106" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6330,12 +6330,12 @@
       <c r="J107" t="inlineStr"/>
       <c r="K107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6383,12 +6383,12 @@
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6436,12 +6436,12 @@
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6489,12 +6489,12 @@
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6542,12 +6542,12 @@
       <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6595,12 +6595,12 @@
       <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6648,12 +6648,12 @@
       <c r="J113" t="inlineStr"/>
       <c r="K113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6701,12 +6701,12 @@
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6754,12 +6754,12 @@
       <c r="J115" t="inlineStr"/>
       <c r="K115" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6807,12 +6807,12 @@
       <c r="J116" t="inlineStr"/>
       <c r="K116" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6860,12 +6860,12 @@
       <c r="J117" t="inlineStr"/>
       <c r="K117" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6913,12 +6913,12 @@
       <c r="J118" t="inlineStr"/>
       <c r="K118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -6970,12 +6970,12 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>12 days, 1:22:26.805603</t>
+          <t>11 days, 1:19:00.980214</t>
         </is>
       </c>
     </row>
@@ -7027,12 +7027,12 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>12 days, 1:22:26.805574</t>
+          <t>11 days, 1:19:00.980177</t>
         </is>
       </c>
     </row>
@@ -7084,12 +7084,12 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>12 days, 1:22:26.805546</t>
+          <t>11 days, 1:19:00.980145</t>
         </is>
       </c>
     </row>
@@ -7137,12 +7137,12 @@
       <c r="J122" t="inlineStr"/>
       <c r="K122" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7190,12 +7190,12 @@
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7243,12 +7243,12 @@
       <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7296,12 +7296,12 @@
       <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7349,12 +7349,12 @@
       <c r="J126" t="inlineStr"/>
       <c r="K126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7402,12 +7402,12 @@
       <c r="J127" t="inlineStr"/>
       <c r="K127" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7455,12 +7455,12 @@
       <c r="J128" t="inlineStr"/>
       <c r="K128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7508,12 +7508,12 @@
       <c r="J129" t="inlineStr"/>
       <c r="K129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7561,12 +7561,12 @@
       <c r="J130" t="inlineStr"/>
       <c r="K130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7614,12 +7614,12 @@
       <c r="J131" t="inlineStr"/>
       <c r="K131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7667,12 +7667,12 @@
       <c r="J132" t="inlineStr"/>
       <c r="K132" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7720,12 +7720,12 @@
       <c r="J133" t="inlineStr"/>
       <c r="K133" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -7777,12 +7777,12 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.805228</t>
+          <t>10 days, 23:49:00.979743</t>
         </is>
       </c>
     </row>
@@ -7834,12 +7834,12 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.805195</t>
+          <t>10 days, 23:49:00.979701</t>
         </is>
       </c>
     </row>
@@ -7891,12 +7891,12 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.805162</t>
+          <t>10 days, 23:49:00.979661</t>
         </is>
       </c>
     </row>
@@ -7948,12 +7948,12 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.805128</t>
+          <t>10 days, 23:49:00.979622</t>
         </is>
       </c>
     </row>
@@ -8005,12 +8005,12 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.805099</t>
+          <t>10 days, 23:49:00.979586</t>
         </is>
       </c>
     </row>
@@ -8062,12 +8062,12 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.805069</t>
+          <t>10 days, 23:49:00.979550</t>
         </is>
       </c>
     </row>
@@ -8119,12 +8119,12 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.805040</t>
+          <t>10 days, 23:49:00.979515</t>
         </is>
       </c>
     </row>
@@ -8176,12 +8176,12 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.805011</t>
+          <t>10 days, 23:49:00.979480</t>
         </is>
       </c>
     </row>
@@ -8233,12 +8233,12 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804982</t>
+          <t>10 days, 23:49:00.979444</t>
         </is>
       </c>
     </row>
@@ -8290,12 +8290,12 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804951</t>
+          <t>10 days, 23:49:00.979407</t>
         </is>
       </c>
     </row>
@@ -8347,12 +8347,12 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804919</t>
+          <t>10 days, 23:49:00.979366</t>
         </is>
       </c>
     </row>
@@ -8404,12 +8404,12 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804886</t>
+          <t>10 days, 23:49:00.979328</t>
         </is>
       </c>
     </row>
@@ -8461,12 +8461,12 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804853</t>
+          <t>10 days, 23:49:00.979288</t>
         </is>
       </c>
     </row>
@@ -8518,12 +8518,12 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804821</t>
+          <t>10 days, 23:49:00.979250</t>
         </is>
       </c>
     </row>
@@ -8575,12 +8575,12 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804787</t>
+          <t>10 days, 23:49:00.979208</t>
         </is>
       </c>
     </row>
@@ -8632,12 +8632,12 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804754</t>
+          <t>10 days, 23:49:00.979169</t>
         </is>
       </c>
     </row>
@@ -8689,12 +8689,12 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804719</t>
+          <t>10 days, 23:49:00.979129</t>
         </is>
       </c>
     </row>
@@ -8746,12 +8746,12 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>11 days, 23:52:26.804684</t>
+          <t>10 days, 23:49:00.979089</t>
         </is>
       </c>
     </row>
@@ -8804,12 +8804,12 @@
       <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -8862,12 +8862,12 @@
       <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -8920,12 +8920,12 @@
       <c r="J154" t="inlineStr"/>
       <c r="K154" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -8978,12 +8978,12 @@
       <c r="J155" t="inlineStr"/>
       <c r="K155" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9036,12 +9036,12 @@
       <c r="J156" t="inlineStr"/>
       <c r="K156" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9094,12 +9094,12 @@
       <c r="J157" t="inlineStr"/>
       <c r="K157" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9152,12 +9152,12 @@
       <c r="J158" t="inlineStr"/>
       <c r="K158" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9210,12 +9210,12 @@
       <c r="J159" t="inlineStr"/>
       <c r="K159" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9268,12 +9268,12 @@
       <c r="J160" t="inlineStr"/>
       <c r="K160" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9326,12 +9326,12 @@
       <c r="J161" t="inlineStr"/>
       <c r="K161" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9388,12 +9388,12 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>11 days, 20:22:26.804357</t>
+          <t>10 days, 20:19:00.978730</t>
         </is>
       </c>
     </row>
@@ -9446,12 +9446,12 @@
       <c r="J163" t="inlineStr"/>
       <c r="K163" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9504,12 +9504,12 @@
       <c r="J164" t="inlineStr"/>
       <c r="K164" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9562,12 +9562,12 @@
       <c r="J165" t="inlineStr"/>
       <c r="K165" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9620,12 +9620,12 @@
       <c r="J166" t="inlineStr"/>
       <c r="K166" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9678,12 +9678,12 @@
       <c r="J167" t="inlineStr"/>
       <c r="K167" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9731,12 +9731,12 @@
       <c r="J168" t="inlineStr"/>
       <c r="K168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9784,12 +9784,12 @@
       <c r="J169" t="inlineStr"/>
       <c r="K169" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9837,12 +9837,12 @@
       <c r="J170" t="inlineStr"/>
       <c r="K170" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9890,12 +9890,12 @@
       <c r="J171" t="inlineStr"/>
       <c r="K171" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9943,12 +9943,12 @@
       <c r="J172" t="inlineStr"/>
       <c r="K172" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -9996,12 +9996,12 @@
       <c r="J173" t="inlineStr"/>
       <c r="K173" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10049,12 +10049,12 @@
       <c r="J174" t="inlineStr"/>
       <c r="K174" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10102,12 +10102,12 @@
       <c r="J175" t="inlineStr"/>
       <c r="K175" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10155,12 +10155,12 @@
       <c r="J176" t="inlineStr"/>
       <c r="K176" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10208,12 +10208,12 @@
       <c r="J177" t="inlineStr"/>
       <c r="K177" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10261,12 +10261,12 @@
       <c r="J178" t="inlineStr"/>
       <c r="K178" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10314,12 +10314,12 @@
       <c r="J179" t="inlineStr"/>
       <c r="K179" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10367,12 +10367,12 @@
       <c r="J180" t="inlineStr"/>
       <c r="K180" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10420,12 +10420,12 @@
       <c r="J181" t="inlineStr"/>
       <c r="K181" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10473,12 +10473,12 @@
       <c r="J182" t="inlineStr"/>
       <c r="K182" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10526,12 +10526,12 @@
       <c r="J183" t="inlineStr"/>
       <c r="K183" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10579,12 +10579,12 @@
       <c r="J184" t="inlineStr"/>
       <c r="K184" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10632,12 +10632,12 @@
       <c r="J185" t="inlineStr"/>
       <c r="K185" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10685,12 +10685,12 @@
       <c r="J186" t="inlineStr"/>
       <c r="K186" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10738,12 +10738,12 @@
       <c r="J187" t="inlineStr"/>
       <c r="K187" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10791,12 +10791,12 @@
       <c r="J188" t="inlineStr"/>
       <c r="K188" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10844,12 +10844,12 @@
       <c r="J189" t="inlineStr"/>
       <c r="K189" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10897,12 +10897,12 @@
       <c r="J190" t="inlineStr"/>
       <c r="K190" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -10950,12 +10950,12 @@
       <c r="J191" t="inlineStr"/>
       <c r="K191" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11003,12 +11003,12 @@
       <c r="J192" t="inlineStr"/>
       <c r="K192" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L192" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11056,12 +11056,12 @@
       <c r="J193" t="inlineStr"/>
       <c r="K193" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11109,12 +11109,12 @@
       <c r="J194" t="inlineStr"/>
       <c r="K194" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11162,12 +11162,12 @@
       <c r="J195" t="inlineStr"/>
       <c r="K195" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11215,12 +11215,12 @@
       <c r="J196" t="inlineStr"/>
       <c r="K196" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11268,12 +11268,12 @@
       <c r="J197" t="inlineStr"/>
       <c r="K197" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11321,12 +11321,12 @@
       <c r="J198" t="inlineStr"/>
       <c r="K198" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11374,12 +11374,12 @@
       <c r="J199" t="inlineStr"/>
       <c r="K199" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11427,12 +11427,12 @@
       <c r="J200" t="inlineStr"/>
       <c r="K200" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11484,12 +11484,12 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>8 days, 23:52:26.803332</t>
+          <t>7 days, 23:49:00.977553</t>
         </is>
       </c>
     </row>
@@ -11537,12 +11537,12 @@
       <c r="J202" t="inlineStr"/>
       <c r="K202" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11590,12 +11590,12 @@
       <c r="J203" t="inlineStr"/>
       <c r="K203" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11643,12 +11643,12 @@
       <c r="J204" t="inlineStr"/>
       <c r="K204" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11696,12 +11696,12 @@
       <c r="J205" t="inlineStr"/>
       <c r="K205" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11749,12 +11749,12 @@
       <c r="J206" t="inlineStr"/>
       <c r="K206" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11802,12 +11802,12 @@
       <c r="J207" t="inlineStr"/>
       <c r="K207" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L207" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11855,12 +11855,12 @@
       <c r="J208" t="inlineStr"/>
       <c r="K208" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11908,12 +11908,12 @@
       <c r="J209" t="inlineStr"/>
       <c r="K209" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -11961,12 +11961,12 @@
       <c r="J210" t="inlineStr"/>
       <c r="K210" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12014,12 +12014,12 @@
       <c r="J211" t="inlineStr"/>
       <c r="K211" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12067,12 +12067,12 @@
       <c r="J212" t="inlineStr"/>
       <c r="K212" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12120,12 +12120,12 @@
       <c r="J213" t="inlineStr"/>
       <c r="K213" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L213" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12173,12 +12173,12 @@
       <c r="J214" t="inlineStr"/>
       <c r="K214" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L214" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12226,12 +12226,12 @@
       <c r="J215" t="inlineStr"/>
       <c r="K215" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L215" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12279,12 +12279,12 @@
       <c r="J216" t="inlineStr"/>
       <c r="K216" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L216" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12332,12 +12332,12 @@
       <c r="J217" t="inlineStr"/>
       <c r="K217" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L217" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12385,12 +12385,12 @@
       <c r="J218" t="inlineStr"/>
       <c r="K218" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12438,12 +12438,12 @@
       <c r="J219" t="inlineStr"/>
       <c r="K219" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L219" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12491,12 +12491,12 @@
       <c r="J220" t="inlineStr"/>
       <c r="K220" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L220" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12544,12 +12544,12 @@
       <c r="J221" t="inlineStr"/>
       <c r="K221" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L221" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12597,12 +12597,12 @@
       <c r="J222" t="inlineStr"/>
       <c r="K222" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12650,12 +12650,12 @@
       <c r="J223" t="inlineStr"/>
       <c r="K223" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L223" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12707,12 +12707,12 @@
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M224" t="inlineStr">
         <is>
-          <t>8 days, 20:22:26.802758</t>
+          <t>7 days, 20:19:00.976843</t>
         </is>
       </c>
     </row>
@@ -12764,12 +12764,12 @@
       </c>
       <c r="K225" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M225" t="inlineStr">
         <is>
-          <t>8 days, 20:22:26.802731</t>
+          <t>7 days, 20:19:00.976806</t>
         </is>
       </c>
     </row>
@@ -12821,12 +12821,12 @@
       </c>
       <c r="K226" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t>8 days, 20:22:26.802703</t>
+          <t>7 days, 20:19:00.976772</t>
         </is>
       </c>
     </row>
@@ -12874,12 +12874,12 @@
       <c r="J227" t="inlineStr"/>
       <c r="K227" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12927,12 +12927,12 @@
       <c r="J228" t="inlineStr"/>
       <c r="K228" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -12980,12 +12980,12 @@
       <c r="J229" t="inlineStr"/>
       <c r="K229" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13033,12 +13033,12 @@
       <c r="J230" t="inlineStr"/>
       <c r="K230" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13086,12 +13086,12 @@
       <c r="J231" t="inlineStr"/>
       <c r="K231" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13139,12 +13139,12 @@
       <c r="J232" t="inlineStr"/>
       <c r="K232" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13192,12 +13192,12 @@
       <c r="J233" t="inlineStr"/>
       <c r="K233" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13245,12 +13245,12 @@
       <c r="J234" t="inlineStr"/>
       <c r="K234" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13298,12 +13298,12 @@
       <c r="J235" t="inlineStr"/>
       <c r="K235" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13351,12 +13351,12 @@
       <c r="J236" t="inlineStr"/>
       <c r="K236" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13404,12 +13404,12 @@
       <c r="J237" t="inlineStr"/>
       <c r="K237" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L237" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13457,12 +13457,12 @@
       <c r="J238" t="inlineStr"/>
       <c r="K238" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13510,12 +13510,12 @@
       <c r="J239" t="inlineStr"/>
       <c r="K239" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13563,12 +13563,12 @@
       <c r="J240" t="inlineStr"/>
       <c r="K240" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13616,12 +13616,12 @@
       <c r="J241" t="inlineStr"/>
       <c r="K241" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13669,12 +13669,12 @@
       <c r="J242" t="inlineStr"/>
       <c r="K242" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13722,12 +13722,12 @@
       <c r="J243" t="inlineStr"/>
       <c r="K243" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13775,12 +13775,12 @@
       <c r="J244" t="inlineStr"/>
       <c r="K244" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13828,12 +13828,12 @@
       <c r="J245" t="inlineStr"/>
       <c r="K245" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13881,12 +13881,12 @@
       <c r="J246" t="inlineStr"/>
       <c r="K246" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13934,12 +13934,12 @@
       <c r="J247" t="inlineStr"/>
       <c r="K247" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -13987,12 +13987,12 @@
       <c r="J248" t="inlineStr"/>
       <c r="K248" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14040,12 +14040,12 @@
       <c r="J249" t="inlineStr"/>
       <c r="K249" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14093,12 +14093,12 @@
       <c r="J250" t="inlineStr"/>
       <c r="K250" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14146,12 +14146,12 @@
       <c r="J251" t="inlineStr"/>
       <c r="K251" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14199,12 +14199,12 @@
       <c r="J252" t="inlineStr"/>
       <c r="K252" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14252,12 +14252,12 @@
       <c r="J253" t="inlineStr"/>
       <c r="K253" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14305,12 +14305,12 @@
       <c r="J254" t="inlineStr"/>
       <c r="K254" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14358,12 +14358,12 @@
       <c r="J255" t="inlineStr"/>
       <c r="K255" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14411,12 +14411,12 @@
       <c r="J256" t="inlineStr"/>
       <c r="K256" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14464,12 +14464,12 @@
       <c r="J257" t="inlineStr"/>
       <c r="K257" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14517,12 +14517,12 @@
       <c r="J258" t="inlineStr"/>
       <c r="K258" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14570,12 +14570,12 @@
       <c r="J259" t="inlineStr"/>
       <c r="K259" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14623,12 +14623,12 @@
       <c r="J260" t="inlineStr"/>
       <c r="K260" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14676,12 +14676,12 @@
       <c r="J261" t="inlineStr"/>
       <c r="K261" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14729,12 +14729,12 @@
       <c r="J262" t="inlineStr"/>
       <c r="K262" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14782,12 +14782,12 @@
       <c r="J263" t="inlineStr"/>
       <c r="K263" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14835,12 +14835,12 @@
       <c r="J264" t="inlineStr"/>
       <c r="K264" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14888,12 +14888,12 @@
       <c r="J265" t="inlineStr"/>
       <c r="K265" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14941,12 +14941,12 @@
       <c r="J266" t="inlineStr"/>
       <c r="K266" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -14994,12 +14994,12 @@
       <c r="J267" t="inlineStr"/>
       <c r="K267" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15047,12 +15047,12 @@
       <c r="J268" t="inlineStr"/>
       <c r="K268" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15100,12 +15100,12 @@
       <c r="J269" t="inlineStr"/>
       <c r="K269" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15153,12 +15153,12 @@
       <c r="J270" t="inlineStr"/>
       <c r="K270" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15206,12 +15206,12 @@
       <c r="J271" t="inlineStr"/>
       <c r="K271" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15263,12 +15263,12 @@
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>4 days, 0:07:26.801586</t>
+          <t>3 days, 0:04:00.975430</t>
         </is>
       </c>
     </row>
@@ -15316,12 +15316,12 @@
       <c r="J273" t="inlineStr"/>
       <c r="K273" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15373,12 +15373,12 @@
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>4 days, 0:07:26.801537</t>
+          <t>3 days, 0:04:00.975369</t>
         </is>
       </c>
     </row>
@@ -15426,12 +15426,12 @@
       <c r="J275" t="inlineStr"/>
       <c r="K275" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15479,12 +15479,12 @@
       <c r="J276" t="inlineStr"/>
       <c r="K276" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15532,12 +15532,12 @@
       <c r="J277" t="inlineStr"/>
       <c r="K277" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15585,12 +15585,12 @@
       <c r="J278" t="inlineStr"/>
       <c r="K278" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15638,12 +15638,12 @@
       <c r="J279" t="inlineStr"/>
       <c r="K279" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15691,12 +15691,12 @@
       <c r="J280" t="inlineStr"/>
       <c r="K280" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15744,12 +15744,12 @@
       <c r="J281" t="inlineStr"/>
       <c r="K281" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15797,12 +15797,12 @@
       <c r="J282" t="inlineStr"/>
       <c r="K282" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15850,12 +15850,12 @@
       <c r="J283" t="inlineStr"/>
       <c r="K283" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15903,12 +15903,12 @@
       <c r="J284" t="inlineStr"/>
       <c r="K284" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -15956,12 +15956,12 @@
       <c r="J285" t="inlineStr"/>
       <c r="K285" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16009,12 +16009,12 @@
       <c r="J286" t="inlineStr"/>
       <c r="K286" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16062,12 +16062,12 @@
       <c r="J287" t="inlineStr"/>
       <c r="K287" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16115,12 +16115,12 @@
       <c r="J288" t="inlineStr"/>
       <c r="K288" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L288" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16168,12 +16168,12 @@
       <c r="J289" t="inlineStr"/>
       <c r="K289" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16221,12 +16221,12 @@
       <c r="J290" t="inlineStr"/>
       <c r="K290" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L290" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16274,12 +16274,12 @@
       <c r="J291" t="inlineStr"/>
       <c r="K291" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L291" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16327,12 +16327,12 @@
       <c r="J292" t="inlineStr"/>
       <c r="K292" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16380,12 +16380,12 @@
       <c r="J293" t="inlineStr"/>
       <c r="K293" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L293" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16433,12 +16433,12 @@
       <c r="J294" t="inlineStr"/>
       <c r="K294" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16486,12 +16486,12 @@
       <c r="J295" t="inlineStr"/>
       <c r="K295" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L295" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16539,12 +16539,12 @@
       <c r="J296" t="inlineStr"/>
       <c r="K296" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16592,12 +16592,12 @@
       <c r="J297" t="inlineStr"/>
       <c r="K297" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16645,12 +16645,12 @@
       <c r="J298" t="inlineStr"/>
       <c r="K298" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16698,12 +16698,12 @@
       <c r="J299" t="inlineStr"/>
       <c r="K299" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16756,12 +16756,12 @@
       <c r="J300" t="inlineStr"/>
       <c r="K300" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L300" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16814,12 +16814,12 @@
       <c r="J301" t="inlineStr"/>
       <c r="K301" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16872,12 +16872,12 @@
       <c r="J302" t="inlineStr"/>
       <c r="K302" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L302" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16930,12 +16930,12 @@
       <c r="J303" t="inlineStr"/>
       <c r="K303" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L303" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -16988,12 +16988,12 @@
       <c r="J304" t="inlineStr"/>
       <c r="K304" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L304" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -17046,12 +17046,12 @@
       <c r="J305" t="inlineStr"/>
       <c r="K305" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L305" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -17104,12 +17104,12 @@
       <c r="J306" t="inlineStr"/>
       <c r="K306" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -17162,12 +17162,12 @@
       <c r="J307" t="inlineStr"/>
       <c r="K307" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -17215,12 +17215,12 @@
       <c r="J308" t="inlineStr"/>
       <c r="K308" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L308" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -17268,12 +17268,12 @@
       <c r="J309" t="inlineStr"/>
       <c r="K309" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -17321,12 +17321,12 @@
       <c r="J310" t="inlineStr"/>
       <c r="K310" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L310" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -17374,12 +17374,12 @@
       <c r="J311" t="inlineStr"/>
       <c r="K311" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -17427,12 +17427,12 @@
       <c r="J312" t="inlineStr"/>
       <c r="K312" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>
@@ -17480,12 +17480,12 @@
       <c r="J313" t="inlineStr"/>
       <c r="K313" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t>08/21/26 10:37 AM</t>
+          <t>08/22/26 10:40 AM</t>
         </is>
       </c>
     </row>

</xml_diff>